<commit_message>
Switch qlCalendarAdvance2(.) vs qlCalendarAdvance(.)
Use more common call with period argument as default.

This is a breaking change.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_bonds.xlsx
+++ b/tests/workbooktests/workbooks/test_bonds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F7C303-12C7-40E2-B231-BB6B8BA4FB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67234E4C-50B7-4352-B9FD-9916C18D493D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3645" yWindow="-19185" windowWidth="30690" windowHeight="16530" firstSheet="7" activeTab="12" xr2:uid="{A8952777-E146-413E-A9B0-D4A573A66C27}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="2" activeTab="2" xr2:uid="{A8952777-E146-413E-A9B0-D4A573A66C27}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabs" sheetId="1" r:id="rId1"/>
@@ -3724,7 +3724,7 @@
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>42</v>
       </c>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>44</v>
       </c>
@@ -3742,17 +3742,17 @@
       </c>
       <c r="C5" s="6"/>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B6" s="11">
-        <f>_xll.qlCalendarAdvance2(B4,B5,"10y","following")</f>
+        <f>_xll.qlCalendarAdvance(B4,B5,"10y","following")</f>
         <v>49317</v>
       </c>
       <c r="C6" s="6"/>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>46</v>
       </c>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="C7" s="6"/>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>47</v>
       </c>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="C8" s="6"/>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>48</v>
       </c>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="C9" s="6"/>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>49</v>
       </c>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6">
         <v>103</v>
@@ -3798,7 +3798,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="6">
         <v>103</v>
@@ -3807,42 +3807,42 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="6">
         <v>103</v>
       </c>
       <c r="C13" s="6"/>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="6">
         <v>103</v>
       </c>
       <c r="C14" s="6"/>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="6">
         <v>102</v>
       </c>
       <c r="C15" s="6"/>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="6">
         <v>102</v>
       </c>
       <c r="C16" s="6"/>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="6">
         <v>102</v>
       </c>
       <c r="C17" s="6"/>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="6">
         <v>102</v>

</xml_diff>

<commit_message>
Add test cases for qlBondSinkingSchedule and qlBondSinkingNotionals.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_bonds.xlsx
+++ b/tests/workbooktests/workbooks/test_bonds.xlsx
@@ -8,25 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB21C28-8590-48C0-AC89-070A617FEADF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D39693-9253-47C1-BCEF-B226CC19D9BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{A8952777-E146-413E-A9B0-D4A573A66C27}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabs" sheetId="1" r:id="rId1"/>
     <sheet name="BondPrice" sheetId="18" r:id="rId2"/>
-    <sheet name="Bond" sheetId="3" r:id="rId3"/>
-    <sheet name="ZeroCouponBond" sheetId="4" r:id="rId4"/>
-    <sheet name="FixedRateBond" sheetId="5" r:id="rId5"/>
-    <sheet name="AmortizingFixedRateBond" sheetId="6" r:id="rId6"/>
-    <sheet name="AmortizingFloatingRateBond" sheetId="7" r:id="rId7"/>
-    <sheet name="FloatingRateBond" sheetId="8" r:id="rId8"/>
-    <sheet name="CmsRateBond" sheetId="9" r:id="rId9"/>
-    <sheet name="AmortizingCmsRateBond" sheetId="10" r:id="rId10"/>
-    <sheet name="Callability" sheetId="21" r:id="rId11"/>
-    <sheet name="CallableFixedRateBond" sheetId="13" r:id="rId12"/>
-    <sheet name="CallableZeroCouponBond" sheetId="14" r:id="rId13"/>
-    <sheet name="CPIBond" sheetId="22" r:id="rId14"/>
+    <sheet name="BondSinkingSchedule_Notionals" sheetId="23" r:id="rId3"/>
+    <sheet name="Bond" sheetId="3" r:id="rId4"/>
+    <sheet name="ZeroCouponBond" sheetId="4" r:id="rId5"/>
+    <sheet name="FixedRateBond" sheetId="5" r:id="rId6"/>
+    <sheet name="AmortizingFixedRateBond" sheetId="6" r:id="rId7"/>
+    <sheet name="AmortizingFloatingRateBond" sheetId="7" r:id="rId8"/>
+    <sheet name="FloatingRateBond" sheetId="8" r:id="rId9"/>
+    <sheet name="CmsRateBond" sheetId="9" r:id="rId10"/>
+    <sheet name="AmortizingCmsRateBond" sheetId="10" r:id="rId11"/>
+    <sheet name="Callability" sheetId="21" r:id="rId12"/>
+    <sheet name="CallableFixedRateBond" sheetId="13" r:id="rId13"/>
+    <sheet name="CallableZeroCouponBond" sheetId="14" r:id="rId14"/>
+    <sheet name="CPIBond" sheetId="22" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="209">
   <si>
     <t>Bond</t>
   </si>
@@ -641,6 +642,33 @@
   </si>
   <si>
     <t>qlCPIBond</t>
+  </si>
+  <si>
+    <t>BondSinkingSchedule_Notionals</t>
+  </si>
+  <si>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>bond_length</t>
+  </si>
+  <si>
+    <t>5Y</t>
+  </si>
+  <si>
+    <t>qlBondSinkingSchedule</t>
+  </si>
+  <si>
+    <t>coupon_rate</t>
+  </si>
+  <si>
+    <t>initial_amount</t>
+  </si>
+  <si>
+    <t>qlBondSinkingNotionals</t>
+  </si>
+  <si>
+    <t>{=qlBondSinkingNotionals(B10;B11;B12;B13)}</t>
   </si>
 </sst>
 </file>
@@ -983,7 +1011,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1244,6 +1272,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1559,7 +1591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1B31AC-6B78-4845-B599-86FA814CB2D7}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="15"/>
@@ -1602,17 +1634,15 @@
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="22"/>
+        <v>200</v>
+      </c>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="27"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="20" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>112</v>
@@ -1622,7 +1652,7 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="21" t="s">
         <v>112</v>
@@ -1632,7 +1662,7 @@
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="20" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>112</v>
@@ -1642,7 +1672,7 @@
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="20" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>112</v>
@@ -1652,7 +1682,7 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="21" t="s">
         <v>112</v>
@@ -1662,7 +1692,7 @@
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C11" s="21" t="s">
         <v>112</v>
@@ -1671,8 +1701,8 @@
       <c r="E11" s="22"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="25" t="s">
-        <v>7</v>
+      <c r="B12" s="20" t="s">
+        <v>6</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>112</v>
@@ -1682,27 +1712,25 @@
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="C13" s="21"/>
+        <v>7</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>112</v>
+      </c>
       <c r="D13" s="21"/>
       <c r="E13" s="22"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="25" t="s">
-        <v>8</v>
+        <v>124</v>
       </c>
       <c r="C14" s="21"/>
-      <c r="D14" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>112</v>
-      </c>
+      <c r="D14" s="21"/>
+      <c r="E14" s="22"/>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="25" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="21" t="s">
@@ -1712,15 +1740,27 @@
         <v>112</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="110" t="s">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C17" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="24"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1732,6 +1772,883 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27515A30-3B44-433D-8DBF-ACC4ED7765FD}">
+  <dimension ref="A1:C74"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.140625" customWidth="1"/>
+    <col min="2" max="2" width="58.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="46.5703125" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2">
+        <v>45659</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2">
+        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>45659</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3">
+        <v>100</v>
+      </c>
+      <c r="C5" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="11">
+        <v>45665</v>
+      </c>
+      <c r="C6" s="11">
+        <v>45665</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="11">
+        <v>49682</v>
+      </c>
+      <c r="C7" s="11">
+        <v>49682</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+      <c r="C9" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="6">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="3" t="str">
+        <f>_xll.qlSchedule(B6,B7,B8,B9,B10,B11,B12,B13)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R14C2Schedule,A</v>
+      </c>
+      <c r="C14" s="3" t="str">
+        <f>_xll.qlSchedule(C6,C7,C8,C9,C10,C11,C12,C13)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R14C3Schedule,A</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6">
+        <v>2</v>
+      </c>
+      <c r="C17" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+      <c r="C19" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="6" t="str">
+        <f>_xll.qlEuribor("3M")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R23C2Euribor,A</v>
+      </c>
+      <c r="C23" s="6" t="str">
+        <f>_xll.qlEuribor("3M")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R23C3Euribor,A</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="6" t="str">
+        <f>_xll.qlFlatForward(B2,0.03,"Actual360","Compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R24C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="C24" s="6" t="str">
+        <f>_xll.qlFlatForward(B2,0.03,"Actual360","Compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R24C3YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>100</v>
+      </c>
+      <c r="B25" s="3" t="str">
+        <f>_xll.qlSwapIndex(B15,B16,B17,B18,B19,B20,B21,B22,B23,B24)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R25C2SwapIndex,A</v>
+      </c>
+      <c r="C25" s="3" t="str">
+        <f>_xll.qlSwapIndex(C15,C16,C17,C18,C19,C20,C21,C22,C23,C24)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R25C3SwapIndex,A</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>84</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" s="3">
+        <v>2</v>
+      </c>
+      <c r="C28" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="3">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" s="3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C30" s="3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="3">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" s="3">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="2">
+        <v>45663</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B36" s="3" t="str">
+        <f>_xll.qlCmsRateBond(B4,B5,B14,B25,B26,B27,B28,B29,B30,B31,B32)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R36C2CmsRateBond,A</v>
+      </c>
+      <c r="C36" s="3" t="str">
+        <f>_xll.qlCmsRateBond(C4,C5,C14,C25,C26,C27,C28,C29,C30,C31,C32,C33,C34,C35)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R36C3CmsRateBond,A</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="3">
+        <f>_xll.qlBondNextCouponRate(B36)</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="3">
+        <f>_xll.qlBondNextCouponRate(C36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" s="3">
+        <f>_xll.qlBondPreviousCouponRate(B36)</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="3">
+        <f>_xll.qlBondPreviousCouponRate(C36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B39" s="2">
+        <f>_xll.qlBondNextCashFlowDate(B36)</f>
+        <v>46030</v>
+      </c>
+      <c r="C39" s="2">
+        <f>_xll.qlBondNextCashFlowDate(C36)</f>
+        <v>46030</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" s="2">
+        <f>_xll.qlBondPreviousCashFlowDate(B36)</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="2">
+        <f>_xll.qlBondPreviousCashFlowDate(C36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B41" s="3">
+        <f>_xll.qlBondSettlementDays(B36)</f>
+        <v>2</v>
+      </c>
+      <c r="C41" s="3">
+        <f>_xll.qlBondSettlementDays(C36)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B42" s="2">
+        <f>_xll.qlBondSettlementDate(B36)</f>
+        <v>45663</v>
+      </c>
+      <c r="C42" s="2">
+        <f>_xll.qlBondSettlementDate(C36)</f>
+        <v>45663</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B43" s="3" t="b">
+        <f>_xll.qlBondIsTradable(B36)</f>
+        <v>1</v>
+      </c>
+      <c r="C43" s="3" t="b">
+        <f>_xll.qlBondIsTradable(C36)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B44" s="2">
+        <f>_xll.qlBondStartDate(B36)</f>
+        <v>45665</v>
+      </c>
+      <c r="C44" s="2">
+        <f>_xll.qlBondStartDate(C36)</f>
+        <v>45665</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45" s="2">
+        <f>_xll.qlBondMaturityDate(B36)</f>
+        <v>49682</v>
+      </c>
+      <c r="C45" s="2">
+        <f>_xll.qlBondMaturityDate(C36)</f>
+        <v>49682</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B46" s="3">
+        <f>_xll.qlBondIssueDate(B36)</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="2">
+        <f>_xll.qlBondIssueDate(C36)</f>
+        <v>45663</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B47" s="3" t="str">
+        <f>_xll.qlBondCashFlows(B36)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R47C2CashFlow,A</v>
+      </c>
+      <c r="C47" s="3" t="str">
+        <f>_xll.qlBondCashFlows(C36)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R47C3CashFlow,A</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B48" s="3" t="str">
+        <f>_xll.qlBondRedemption(B36)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R48C2CashFlow,A</v>
+      </c>
+      <c r="C48" s="3" t="str">
+        <f>_xll.qlBondRedemption(C36)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R48C3CashFlow,A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="3" t="str">
+        <f>_xll.qlBondRedemptions(B36)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R49C2CashFlow,A</v>
+      </c>
+      <c r="C49" s="3" t="str">
+        <f>_xll.qlBondRedemptions(C36)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R49C3CashFlow,A</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B50" s="3" t="str">
+        <f>_xll.qlBondCalendar(B36)</f>
+        <v>TARGET</v>
+      </c>
+      <c r="C50" s="3" t="str">
+        <f>_xll.qlBondCalendar(C36)</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B51" s="3">
+        <f>_xll.qlBondNotional(B36)</f>
+        <v>100</v>
+      </c>
+      <c r="C51" s="3">
+        <f>_xll.qlBondNotional(C36)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="3">
+        <f>_xll.qlBondNotionals(B36)</f>
+        <v>100</v>
+      </c>
+      <c r="C52" s="3">
+        <f>_xll.qlBondNotionals(C36)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="3" t="str">
+        <f>_xll.qlFlatForward(B2,0.03,"actual360","compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R53C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="C53" s="3" t="str">
+        <f>_xll.qlFlatForward(B2,0.03,"actual360","compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R53C3YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B54" s="3" t="str">
+        <f>_xll.qlDiscountingBondEngine(B53)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R54C2DiscountingBondEngine,A</v>
+      </c>
+      <c r="C54" s="3" t="str">
+        <f>_xll.qlDiscountingBondEngine(C53)</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R54C3DiscountingBondEngine,A</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B55" s="3" t="b">
+        <f>_xll.qlInstrumentSetPricingEngine(B36,B54)</f>
+        <v>1</v>
+      </c>
+      <c r="C55" s="3" t="b">
+        <f>_xll.qlInstrumentSetPricingEngine(C36,C54)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B56" s="9">
+        <f>_xll.qlBondCleanPrice(B36,B55)</f>
+        <v>71.629228665106581</v>
+      </c>
+      <c r="C56" s="9">
+        <f>_xll.qlBondCleanPrice(C36,C55)</f>
+        <v>85.955074398127891</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57" s="9">
+        <v>2.9888064241409301E-2</v>
+      </c>
+      <c r="C57" s="9">
+        <v>2.9888064241409301E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B58" s="9">
+        <f>_xll.qlBondCleanPrice2(B36,B57,"actual360","continuous")</f>
+        <v>71.629224757480401</v>
+      </c>
+      <c r="C58" s="9">
+        <f>_xll.qlBondCleanPrice2(C36,C57,"actual360","continuous")</f>
+        <v>85.955069708976481</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B59" s="9">
+        <f>_xll.qlBondDirtyPrice(B36,B55)</f>
+        <v>71.629228665106581</v>
+      </c>
+      <c r="C59" s="9">
+        <f>_xll.qlBondDirtyPrice(C36,C55)</f>
+        <v>85.955074398127891</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B60" s="9">
+        <f>_xll.qlBondDirtyPrice2(B36,B57,"actual360","CONTINUOUS","annual")</f>
+        <v>71.629224757480401</v>
+      </c>
+      <c r="C60" s="9">
+        <f>_xll.qlBondDirtyPrice2(C36,C57,"actual360","CONTINUOUS","annual")</f>
+        <v>85.955069708976481</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B61" s="9">
+        <f>_xll.qlBondYield(B36,"actual360","CONTINUOUS","annual",,,B55)</f>
+        <v>2.9888064241409308E-2</v>
+      </c>
+      <c r="C61" s="9">
+        <f>_xll.qlBondYield(C36,"actual360","CONTINUOUS","annual",,,C55)</f>
+        <v>2.9888064241409308E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B62" s="9" t="str">
+        <f>_xll.qlBondPrice(B56,"clean")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R62C2BondPrice,A</v>
+      </c>
+      <c r="C62" s="9" t="str">
+        <f>_xll.qlBondPrice(C56,"clean")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R62C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B63" s="9">
+        <f>_xll.qlBondYield2(B36,B62,"actual360","CONTINUOUS","annual")</f>
+        <v>2.9888064241409308E-2</v>
+      </c>
+      <c r="C63" s="9">
+        <f>_xll.qlBondYield2(C36,C62,"actual360","CONTINUOUS","annual")</f>
+        <v>2.9888064241409308E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B64" s="2">
+        <v>45667</v>
+      </c>
+      <c r="C64" s="2">
+        <v>45667</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B65" s="9">
+        <f>_xll.qlBondAccruedAmount(B36,B64)</f>
+        <v>0</v>
+      </c>
+      <c r="C65" s="9">
+        <f>_xll.qlBondAccruedAmount(C36,C64)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B66" s="9">
+        <f>_xll.qlBondSettlementValue(B36,B55)</f>
+        <v>71.629228665106581</v>
+      </c>
+      <c r="C66" s="9">
+        <f>_xll.qlBondSettlementValue(C36,C55)</f>
+        <v>85.955074398127891</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B67" s="9">
+        <f>_xll.qlBondSettlementValue2(B36,B56)</f>
+        <v>71.629228665106581</v>
+      </c>
+      <c r="C67" s="9">
+        <f>_xll.qlBondSettlementValue2(C36,C56)</f>
+        <v>85.955074398127891</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B68" s="9" t="str">
+        <f>_xll.qlFlatForward($B$1,0.03,"actual365fixed")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R68C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="C68" s="9" t="str">
+        <f>_xll.qlFlatForward($B$1,0.03,"actual365fixed")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R68C3YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B69" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C69" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B74" s="3">
+        <f>_xll.qlBondCleanPriceFromZSpread(B36,B68,B69,B70,B71,B72)</f>
+        <v>68.138537120691339</v>
+      </c>
+      <c r="C74" s="3">
+        <f>_xll.qlBondCleanPriceFromZSpread(C36,C68,C69,C70,C71,C72)</f>
+        <v>81.766244544829618</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28ABD84F-1436-4AE1-BC17-091C65B56114}">
   <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2613,7 +3530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F09BC366-53EA-43EA-8BCB-0489C1B271E0}">
   <dimension ref="A3:B12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2692,7 +3609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F0A1FE9-B1FE-4762-AEA9-E4B3F6C519F7}">
   <dimension ref="A1:C219"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4470,7 +5387,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D4EF9C2-FD4D-4E7F-8154-C8E782972C6B}">
   <dimension ref="A1:C206"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6102,7 +7019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5B778A-9E41-4D83-BBAD-BAE5A92DD1A2}">
   <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7122,6 +8039,128 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2242D3EA-26F0-4B90-9FC1-2485363E0315}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.7109375" style="3" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2">
+        <v>45659</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2">
+        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>45659</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="119" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="2">
+        <v>45659</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="119" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="119" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="119" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="3" t="str">
+        <f>_xll.qlBondSinkingSchedule(B4,B5,B6,B7)</f>
+        <v>欣[test_bonds.xlsx]BondSinkingSchedule_Notionals!R8C2Schedule,A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="119" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="119" t="s">
+        <v>189</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="119" t="s">
+        <v>205</v>
+      </c>
+      <c r="B12" s="3">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="119" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="3">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B14" s="3">
+        <f>_xll.qlBondSinkingNotionals(B10,B11,B12,B13)</f>
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="120" t="s">
+        <v>208</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8683113-FD1C-4D88-8D42-F7763B404E4F}">
   <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7763,7 +8802,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA0BDDB4-6035-4089-86B1-6246F3228CBC}">
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8355,7 +9394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EB77E5-949B-439C-BFA2-575F2A710E3C}">
   <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9110,7 +10149,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{303A5445-988F-4FD7-9234-8C10A40DEB2F}">
   <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9965,7 +11004,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F76F30CA-2F79-453E-B116-2A48310E361D}">
   <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10778,7 +11817,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05025377-E5EA-48F0-BE68-1C47A2C5C8E6}">
   <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11558,881 +12597,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27515A30-3B44-433D-8DBF-ACC4ED7765FD}">
-  <dimension ref="A1:C74"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="46.140625" customWidth="1"/>
-    <col min="2" max="2" width="58.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="46.5703125" style="3" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="2">
-        <v>45659</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="2">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45659</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="3">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="3">
-        <v>100</v>
-      </c>
-      <c r="C5" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="11">
-        <v>45665</v>
-      </c>
-      <c r="C6" s="11">
-        <v>45665</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="11">
-        <v>49682</v>
-      </c>
-      <c r="C7" s="11">
-        <v>49682</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C9" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="6">
-        <v>0</v>
-      </c>
-      <c r="C13" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="3" t="str">
-        <f>_xll.qlSchedule(B6,B7,B8,B9,B10,B11,B12,B13)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R14C2Schedule,A</v>
-      </c>
-      <c r="C14" s="3" t="str">
-        <f>_xll.qlSchedule(C6,C7,C8,C9,C10,C11,C12,C13)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R14C3Schedule,A</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="6">
-        <v>2</v>
-      </c>
-      <c r="C17" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C19" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B23" s="6" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R23C2Euribor,A</v>
-      </c>
-      <c r="C23" s="6" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R23C3Euribor,A</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B24" s="6" t="str">
-        <f>_xll.qlFlatForward(B2,0.03,"Actual360","Compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R24C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C24" s="6" t="str">
-        <f>_xll.qlFlatForward(B2,0.03,"Actual360","Compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R24C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>100</v>
-      </c>
-      <c r="B25" s="3" t="str">
-        <f>_xll.qlSwapIndex(B15,B16,B17,B18,B19,B20,B21,B22,B23,B24)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R25C2SwapIndex,A</v>
-      </c>
-      <c r="C25" s="3" t="str">
-        <f>_xll.qlSwapIndex(C15,C16,C17,C18,C19,C20,C21,C22,C23,C24)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R25C3SwapIndex,A</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>67</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>84</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>90</v>
-      </c>
-      <c r="B28" s="3">
-        <v>2</v>
-      </c>
-      <c r="C28" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="B29" s="3">
-        <v>0</v>
-      </c>
-      <c r="C29" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>92</v>
-      </c>
-      <c r="B30" s="3">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C30" s="3">
-        <v>3.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B31" s="3">
-        <v>0</v>
-      </c>
-      <c r="C31" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B32" s="3">
-        <v>0</v>
-      </c>
-      <c r="C32" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>95</v>
-      </c>
-      <c r="C33" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="3">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C35" s="2">
-        <v>45663</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B36" s="3" t="str">
-        <f>_xll.qlCmsRateBond(B4,B5,B14,B25,B26,B27,B28,B29,B30,B31,B32)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R36C2CmsRateBond,A</v>
-      </c>
-      <c r="C36" s="3" t="str">
-        <f>_xll.qlCmsRateBond(C4,C5,C14,C25,C26,C27,C28,C29,C30,C31,C32,C33,C34,C35)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R36C3CmsRateBond,A</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" s="3">
-        <f>_xll.qlBondNextCouponRate(B36)</f>
-        <v>0</v>
-      </c>
-      <c r="C37" s="3">
-        <f>_xll.qlBondNextCouponRate(C36)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B38" s="3">
-        <f>_xll.qlBondPreviousCouponRate(B36)</f>
-        <v>0</v>
-      </c>
-      <c r="C38" s="3">
-        <f>_xll.qlBondPreviousCouponRate(C36)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B39" s="2">
-        <f>_xll.qlBondNextCashFlowDate(B36)</f>
-        <v>46030</v>
-      </c>
-      <c r="C39" s="2">
-        <f>_xll.qlBondNextCashFlowDate(C36)</f>
-        <v>46030</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B40" s="2">
-        <f>_xll.qlBondPreviousCashFlowDate(B36)</f>
-        <v>0</v>
-      </c>
-      <c r="C40" s="2">
-        <f>_xll.qlBondPreviousCashFlowDate(C36)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B41" s="3">
-        <f>_xll.qlBondSettlementDays(B36)</f>
-        <v>2</v>
-      </c>
-      <c r="C41" s="3">
-        <f>_xll.qlBondSettlementDays(C36)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B42" s="2">
-        <f>_xll.qlBondSettlementDate(B36)</f>
-        <v>45663</v>
-      </c>
-      <c r="C42" s="2">
-        <f>_xll.qlBondSettlementDate(C36)</f>
-        <v>45663</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B43" s="3" t="b">
-        <f>_xll.qlBondIsTradable(B36)</f>
-        <v>1</v>
-      </c>
-      <c r="C43" s="3" t="b">
-        <f>_xll.qlBondIsTradable(C36)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B44" s="2">
-        <f>_xll.qlBondStartDate(B36)</f>
-        <v>45665</v>
-      </c>
-      <c r="C44" s="2">
-        <f>_xll.qlBondStartDate(C36)</f>
-        <v>45665</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B45" s="2">
-        <f>_xll.qlBondMaturityDate(B36)</f>
-        <v>49682</v>
-      </c>
-      <c r="C45" s="2">
-        <f>_xll.qlBondMaturityDate(C36)</f>
-        <v>49682</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B46" s="3">
-        <f>_xll.qlBondIssueDate(B36)</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="2">
-        <f>_xll.qlBondIssueDate(C36)</f>
-        <v>45663</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B47" s="3" t="str">
-        <f>_xll.qlBondCashFlows(B36)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R47C2CashFlow,A</v>
-      </c>
-      <c r="C47" s="3" t="str">
-        <f>_xll.qlBondCashFlows(C36)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R47C3CashFlow,A</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B48" s="3" t="str">
-        <f>_xll.qlBondRedemption(B36)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R48C2CashFlow,A</v>
-      </c>
-      <c r="C48" s="3" t="str">
-        <f>_xll.qlBondRedemption(C36)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R48C3CashFlow,A</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49" s="3" t="str">
-        <f>_xll.qlBondRedemptions(B36)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R49C2CashFlow,A</v>
-      </c>
-      <c r="C49" s="3" t="str">
-        <f>_xll.qlBondRedemptions(C36)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R49C3CashFlow,A</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B50" s="3" t="str">
-        <f>_xll.qlBondCalendar(B36)</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C50" s="3" t="str">
-        <f>_xll.qlBondCalendar(C36)</f>
-        <v>TARGET</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B51" s="3">
-        <f>_xll.qlBondNotional(B36)</f>
-        <v>100</v>
-      </c>
-      <c r="C51" s="3">
-        <f>_xll.qlBondNotional(C36)</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52" s="3">
-        <f>_xll.qlBondNotionals(B36)</f>
-        <v>100</v>
-      </c>
-      <c r="C52" s="3">
-        <f>_xll.qlBondNotionals(C36)</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B53" s="3" t="str">
-        <f>_xll.qlFlatForward(B2,0.03,"actual360","compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R53C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C53" s="3" t="str">
-        <f>_xll.qlFlatForward(B2,0.03,"actual360","compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R53C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="B54" s="3" t="str">
-        <f>_xll.qlDiscountingBondEngine(B53)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R54C2DiscountingBondEngine,A</v>
-      </c>
-      <c r="C54" s="3" t="str">
-        <f>_xll.qlDiscountingBondEngine(C53)</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R54C3DiscountingBondEngine,A</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B55" s="3" t="b">
-        <f>_xll.qlInstrumentSetPricingEngine(B36,B54)</f>
-        <v>1</v>
-      </c>
-      <c r="C55" s="3" t="b">
-        <f>_xll.qlInstrumentSetPricingEngine(C36,C54)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B56" s="9">
-        <f>_xll.qlBondCleanPrice(B36,B55)</f>
-        <v>71.629228665106581</v>
-      </c>
-      <c r="C56" s="9">
-        <f>_xll.qlBondCleanPrice(C36,C55)</f>
-        <v>85.955074398127891</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="B57" s="9">
-        <v>2.9888064241409301E-2</v>
-      </c>
-      <c r="C57" s="9">
-        <v>2.9888064241409301E-2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B58" s="9">
-        <f>_xll.qlBondCleanPrice2(B36,B57,"actual360","continuous")</f>
-        <v>71.629224757480401</v>
-      </c>
-      <c r="C58" s="9">
-        <f>_xll.qlBondCleanPrice2(C36,C57,"actual360","continuous")</f>
-        <v>85.955069708976481</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B59" s="9">
-        <f>_xll.qlBondDirtyPrice(B36,B55)</f>
-        <v>71.629228665106581</v>
-      </c>
-      <c r="C59" s="9">
-        <f>_xll.qlBondDirtyPrice(C36,C55)</f>
-        <v>85.955074398127891</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B60" s="9">
-        <f>_xll.qlBondDirtyPrice2(B36,B57,"actual360","CONTINUOUS","annual")</f>
-        <v>71.629224757480401</v>
-      </c>
-      <c r="C60" s="9">
-        <f>_xll.qlBondDirtyPrice2(C36,C57,"actual360","CONTINUOUS","annual")</f>
-        <v>85.955069708976481</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B61" s="9">
-        <f>_xll.qlBondYield(B36,"actual360","CONTINUOUS","annual",,,B55)</f>
-        <v>2.9888064241409308E-2</v>
-      </c>
-      <c r="C61" s="9">
-        <f>_xll.qlBondYield(C36,"actual360","CONTINUOUS","annual",,,C55)</f>
-        <v>2.9888064241409308E-2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B62" s="9" t="str">
-        <f>_xll.qlBondPrice(B56,"clean")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R62C2BondPrice,A</v>
-      </c>
-      <c r="C62" s="9" t="str">
-        <f>_xll.qlBondPrice(C56,"clean")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R62C3BondPrice,A</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B63" s="9">
-        <f>_xll.qlBondYield2(B36,B62,"actual360","CONTINUOUS","annual")</f>
-        <v>2.9888064241409308E-2</v>
-      </c>
-      <c r="C63" s="9">
-        <f>_xll.qlBondYield2(C36,C62,"actual360","CONTINUOUS","annual")</f>
-        <v>2.9888064241409308E-2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B64" s="2">
-        <v>45667</v>
-      </c>
-      <c r="C64" s="2">
-        <v>45667</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B65" s="9">
-        <f>_xll.qlBondAccruedAmount(B36,B64)</f>
-        <v>0</v>
-      </c>
-      <c r="C65" s="9">
-        <f>_xll.qlBondAccruedAmount(C36,C64)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B66" s="9">
-        <f>_xll.qlBondSettlementValue(B36,B55)</f>
-        <v>71.629228665106581</v>
-      </c>
-      <c r="C66" s="9">
-        <f>_xll.qlBondSettlementValue(C36,C55)</f>
-        <v>85.955074398127891</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B67" s="9">
-        <f>_xll.qlBondSettlementValue2(B36,B56)</f>
-        <v>71.629228665106581</v>
-      </c>
-      <c r="C67" s="9">
-        <f>_xll.qlBondSettlementValue2(C36,C56)</f>
-        <v>85.955074398127891</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="B68" s="9" t="str">
-        <f>_xll.qlFlatForward($B$1,0.03,"actual365fixed")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R68C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C68" s="9" t="str">
-        <f>_xll.qlFlatForward($B$1,0.03,"actual365fixed")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R68C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="B69" s="9">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C69" s="9">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="B70" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="C70" s="9" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="C71" s="9" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="B72" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="C72" s="9" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="B74" s="3">
-        <f>_xll.qlBondCleanPriceFromZSpread(B36,B68,B69,B70,B71,B72)</f>
-        <v>68.138537120691339</v>
-      </c>
-      <c r="C74" s="3">
-        <f>_xll.qlBondCleanPriceFromZSpread(C36,C68,C69,C70,C71,C72)</f>
-        <v>81.766244544829618</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>